<commit_message>
Small REGF1 tuning change
</commit_message>
<xml_diff>
--- a/ID_code/ANDES_Dutch_2035_mpc_ID.xlsx
+++ b/ID_code/ANDES_Dutch_2035_mpc_ID.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piete\Documents\pieter\school\studie\Master\THESIS\CODE\HPvanRhee_MScThesis_Documentation\ID_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728EFB8E-D5B0-421B-94F3-04B6AFEEC0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57003DA3-BCC6-4F91-989B-97014854C269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27060" yWindow="2025" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24270" yWindow="2580" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -7783,10 +7783,10 @@
       </c>
       <c r="Z2">
         <f>AA2/2</f>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="AA2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AB2">
         <v>0.33</v>
@@ -7856,10 +7856,10 @@
       </c>
       <c r="Z3">
         <f>AA3/2</f>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="AA3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AB3">
         <v>0.33</v>

</xml_diff>